<commit_message>
Replace sample outputs with Sea Limited run
</commit_message>
<xml_diff>
--- a/hpi_scraper/Firmographic/apollo/apollo_api_report.xlsx
+++ b/hpi_scraper/Firmographic/apollo/apollo_api_report.xlsx
@@ -556,12 +556,12 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>1 organization enrich API units consumed today; 1 consumed this hour</t>
+          <t>2 organization enrich API units consumed today; 2 consumed this hour</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>organization enrich day 600 consumed 1 left 599; hour 200 consumed 1 left 199; minute 50 left 49</t>
+          <t>organization enrich day 600 consumed 2 left 598; hour 200 consumed 2 left 198; minute 50 left 49</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>1.784 avg</t>
+          <t>1.419 avg</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>Y - number_of_sites_locations_sg_global; funding_total</t>
+          <t>Y - website_domain; revenue_or_revenue_band; number_of_sites_locations_sg_global; ownership_type; funding_total</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Refresh FullEnrich contact output and polish reports
</commit_message>
<xml_diff>
--- a/hpi_scraper/Firmographic/apollo/apollo_api_report.xlsx
+++ b/hpi_scraper/Firmographic/apollo/apollo_api_report.xlsx
@@ -449,15 +449,15 @@
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="72" customWidth="1" min="5" max="5"/>
+    <col width="72" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="55" customWidth="1" min="12" max="12"/>
-    <col width="55" customWidth="1" min="13" max="13"/>
+    <col width="72" customWidth="1" min="12" max="12"/>
+    <col width="72" customWidth="1" min="13" max="13"/>
     <col width="24" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -556,23 +556,19 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>2 organization enrich API units consumed today; 2 consumed this hour</t>
+          <t>2 Apollo organization-enrich units consumed in the account-day counter for this Sea Limited check.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>organization enrich day 600 consumed 2 left 598; hour 200 consumed 2 left 198; minute 50 left 49</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
+          <t>Apollo usage endpoint showed day 600 limit / 598 remaining, hour 200 / 198 remaining, minute bucket available at run time.</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
@@ -584,19 +580,17 @@
           <t>200:1</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="K2" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>Y - website_domain; revenue_or_revenue_band; number_of_sites_locations_sg_global; ownership_type; funding_total</t>
+          <t>Partial - Apollo returned company identity, LinkedIn, headcount, industry, HQ and founded year; revenue band, site count and funding were not present.</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Apollo enrichment does not return funding_total for these public companies. Apollo also returns retail_location_count, not a full SG/global site-count field; zero retail counts are treated as unavailable, not as real zero locations.</t>
+          <t>Use Coresignal as the stronger firmographic source for domain and company profile completeness. Apollo did not expose funding or a reliable location/site-count field in this response.</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">

</xml_diff>